<commit_message>
Report: tabulky a grafy číslované místo písmen, kontrola odkazů
Za 26. tabulkou vznikal odkaz „tab. [“ (písmena A–Z došla). Tabulky a grafy se teď číslují
(tab. 1, graf 1), každý typ zvlášť, průběžně v pořadí PDF.
- report_pdf: Sestava.cislo_tab/cislo_graf, klíč „cislo“; kontrola_odkazu před sazbou
  (prázdný či nedokončený odkaz, odkaz na neexistující tabulku nebo graf = chyba sazby)
- šablona Typst: Tabulka N / Graf N
- report_kontrola: odkazy „tab. N“, „Tabulka N“, „graf N“ nejsou čísla z dat
- report: slovní odkaz „tab. přepočtu“ → „viz tabulka přepočtu“
- testy TestOdkazy; pilot F × Liberecký kraj přepočítaný; archivní výstupy beze změny
- docs/report_osnova.md: pravidlo číslování

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U7RRgPmyDg48516c6s7TrK
</commit_message>
<xml_diff>
--- a/reporty/vystupy/F__CZ051__2026-10-15/priloha.xlsx
+++ b/reporty/vystupy/F__CZ051__2026-10-15/priloha.xlsx
@@ -3804,7 +3804,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>přidaná hodnota na úrovni SBS (vstup modelu, tab. přepočtu); obrat = modelový odhad</t>
+          <t>přidaná hodnota na úrovni SBS (vstup modelu, viz tabulka přepočtu); obrat = modelový odhad</t>
         </is>
       </c>
     </row>
@@ -12569,7 +12569,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-19T09:35:12+00:00</t>
+          <t>2026-10-19T09:48:52+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pilot F × Liberecký kraj (CZ-NACE 2025): schválený výklad analytika a vysázené PDF
- výklad analytika: Shrnutí, Modelové odhady a upravené pododdíly Struktura, Ekonomický profil
  a Dynamika vložené beze změny znění (Shrnutí jen ve formátu bodů souboru)
- reporty/ukazky/F__CZ051__2026-10-15: report.pdf (31 stran, --vyklad-schvalen), priloha.xlsx,
  zjisteni.json; kontrola výstupu, čísel v PDF, odkazů a zakázaných slov prošla
- strojová poznámka modelu: „podíl největších firem“ → „podíl největších subjektů“ (rozhodnutí 1)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U7RRgPmyDg48516c6s7TrK
</commit_message>
<xml_diff>
--- a/reporty/vystupy/F__CZ051__2026-10-15/priloha.xlsx
+++ b/reporty/vystupy/F__CZ051__2026-10-15/priloha.xlsx
@@ -4195,7 +4195,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Koncentrace podle velikostních tříd, ne podle jednotlivých subjektů; podíl největších firem by vyžadoval účetní závěrky (Sbírka listin).</t>
+          <t>Koncentrace podle velikostních tříd, ne podle jednotlivých subjektů; podíl největších subjektů by vyžadoval účetní závěrky (Sbírka listin).</t>
         </is>
       </c>
     </row>
@@ -12569,7 +12569,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-19T09:48:52+00:00</t>
+          <t>2026-10-19T10:09:05+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>